<commit_message>
Fix category validation and update scraped data
</commit_message>
<xml_diff>
--- a/output/products.xlsx
+++ b/output/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,44 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>Books to Scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>The Light of the Fireflies</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://books.toscrape.com/catalogue/the-light-of-the-fireflies_71/index.html</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>A haunting and hopeful tale of discovering light in even the darkest of places.For his whole life, the boy has lived underground, in a basement with his parents, grandmother, sister, and brother. Before he was born, his family was disfigured by a fire. His sister wears a white mask to cover her burns.He spends his hours with his cactus, reading his book on insects, or touching the one ray of sunlight that filters in through a crack in the ceiling. Ever since his sister had a baby, everyone’s been acting very strangely. The boy begins to wonder why they never say who the father is, about what happened before his own birth, about why they’re shut away.A few days ago, some fireflies arrived in the basement. His grandma said, There’s no creature more amazing than one that can make its own light. That light makes the boy want to escape, to know the outside world. Problem is, all the doors are locked. And he doesn’t know how to get out.…</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Books to Scrape</t>
         </is>

</xml_diff>

<commit_message>
Refactor, polish, test, and complete E-Commerce Product Data Web Scraper (Internship Task 11)
</commit_message>
<xml_diff>
--- a/output/products.xlsx
+++ b/output/products.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5E7EB"/>
+        <bgColor rgb="00E5E7EB"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,44 +430,54 @@
   </sheetPr>
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>availability</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
@@ -461,14 +486,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A Light in the Attic</t>
+          <t>Lenovo Essential 15.6" FHD Everyday Laptop, Intel Processor, 128GB Storage | Long Battery Life, Anti-Glare Display, Office 365, Copilot AI, WiFi 6, Bluetooth 5.2, USB-C, Win 11</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>51.77</v>
+        <v>349.99</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -477,36 +502,36 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://books.toscrape.com/catalogue/a-light-in-the-attic_1000/index.html</t>
+          <t>https://www.amazon.com/dp/B0HDC9Q8Q6</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Electronics / General</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>It's hard to imagine a world without A Light in the Attic. This now-classic collection of poetry and drawings from Shel Silverstein celebrates its 20th anniversary with this special edition. Silverstein's humorous and creative verse can amuse the dowdiest of readers. Lemon-faced adults and fidgety kids sit still and read these rhythmic words and laugh and smile and love that Silverstein. Need proof of his genius? RockabyeRockabye baby, in the treetopDon't you know a treetopIs no safe place to rock?And who put you up there,And your cradle, too?Baby, I think someone down here'sGot it in for you. Shel, you never sounded so good.</t>
+          <t>FREE delivery Thu, Sep 10Or fastest delivery Wed, Sep 9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Books to Scrape</t>
+          <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>All the Light We Cannot See</t>
+          <t>HP New Everyday Slim Laptop, 2026 Edition, AMD High Performance Processor, 4GB DDR5 RAM, 128GB SSD, Long Battery Life, Windows 11</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29.87</v>
+        <v>299.95</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -515,36 +540,36 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://books.toscrape.com/catalogue/all-the-light-we-cannot-see_660/index.html</t>
+          <t>https://www.amazon.com/dp/B0H7M7M6Z5</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Historical</t>
+          <t>Electronics / General</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>WINNER OF THE PULITZER PRIZEFrom the highly acclaimed, multiple award-winning Anthony Doerr, the beautiful, stunningly ambitious instant New York Times bestseller about a blind French girl and a German boy whose paths collide in occupied France as both try to survive the devastation of World War II.Marie-Laure lives with her father in Paris near the Museum of Natural History, where he works as the master of its thousands of locks. When she is six, Marie-Laure goes blind and her father builds a perfect miniature of their neighborhood so she can memorize it by touch and navigate her way home. When she is twelve, the Nazis occupy Paris and father and daughter flee to the walled citadel of Saint-Malo, where Marie-Laure’s reclusive great-uncle lives in a tall house by the sea. With them they carry what might be the museum’s most valuable and dangerous jewel.In a mining town in Germany, the orphan Werner grows up with his younger sister, enchanted by a crude radio they find. Werner becomes an expert at building and fixing these crucial new instruments, a talent that wins him a place at a brutal academy for Hitler Youth, then a special assignment to track the resistance. More and more aware of the human cost of his intelligence, Werner travels through the heart of the war and, finally, into Saint-Malo, where his story and Marie-Laure’s converge.Doerr’s “stunning sense of physical detail and gorgeous metaphors” (San Francisco Chronicle) are dazzling. Deftly interweaving the lives of Marie-Laure and Werner, he illuminates the ways, against all odds, people try to be good to one another. Ten years in the writing, a National Book Award finalist, All the Light We Cannot See is a magnificent, deeply moving novel from a writer “whose sentences never fail to thrill” (Los Angeles Times).</t>
+          <t>FREE delivery Wed, Sep 9</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Books to Scrape</t>
+          <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The Light of the Fireflies</t>
+          <t>15.6'' AI Laptop with Office 365 12GB RAM 256GB SSD Win 11 Laptops | 7000mAh Battery, IPS FHD, 180°Viewing, Quad-Core Processor, Type-C, WiFi5, Portable Thin Business Student Laptops, Light Gray</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54.43</v>
+        <v>329.98</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>4.4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -553,22 +578,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://books.toscrape.com/catalogue/the-light-of-the-fireflies_71/index.html</t>
+          <t>https://www.amazon.com/dp/B0H94LG15F</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Electronics / General</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>A haunting and hopeful tale of discovering light in even the darkest of places.For his whole life, the boy has lived underground, in a basement with his parents, grandmother, sister, and brother. Before he was born, his family was disfigured by a fire. His sister wears a white mask to cover her burns.He spends his hours with his cactus, reading his book on insects, or touching the one ray of sunlight that filters in through a crack in the ceiling. Ever since his sister had a baby, everyone’s been acting very strangely. The boy begins to wonder why they never say who the father is, about what happened before his own birth, about why they’re shut away.A few days ago, some fireflies arrived in the basement. His grandma said, There’s no creature more amazing than one that can make its own light. That light makes the boy want to escape, to know the outside world. Problem is, all the doors are locked. And he doesn’t know how to get out.…</t>
+          <t>Join Prime to get FREE delivery Tomorrow, Sep 7Or Non-members get FREE delivery Fri, Sep 11</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Books to Scrape</t>
+          <t>Amazon</t>
         </is>
       </c>
     </row>

</xml_diff>